<commit_message>
Update button and other documents
</commit_message>
<xml_diff>
--- a/Non Code Items/Documents/1180 Experience Map.xlsx
+++ b/Non Code Items/Documents/1180 Experience Map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30602"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ncstudents-my.sharepoint.com/personal/ehalilovic2_ncstudents_niagaracollege_ca/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ncstudents-my.sharepoint.com/personal/smutrux1_ncstudents_niagaracollege_ca/Documents/Course Files/Term 3/Prog 1180/Project/prog1180/Non Code Items/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C1C4769-0E42-49EA-92C3-1DA2013C5856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{0C1C4769-0E42-49EA-92C3-1DA2013C5856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71AC869E-007A-44BB-AEC1-D97CB23B3E66}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6585" yWindow="6585" windowWidth="43200" windowHeight="23445" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -172,7 +172,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -353,9 +353,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -393,7 +393,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -499,7 +499,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -641,7 +641,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -650,7 +650,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.28515625" customWidth="1"/>
@@ -662,7 +662,7 @@
     <col min="8" max="8" width="26.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
@@ -672,7 +672,7 @@
       <c r="E1" s="18"/>
       <c r="F1" s="18"/>
     </row>
-    <row r="2" spans="1:19" ht="15.95">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
@@ -692,7 +692,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="32.1">
+    <row r="3" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
@@ -712,7 +712,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="144">
+    <row r="4" spans="1:19" ht="150" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>13</v>
       </c>
@@ -742,7 +742,7 @@
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
     </row>
-    <row r="5" spans="1:19" ht="128.1">
+    <row r="5" spans="1:19" ht="150" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>19</v>
       </c>
@@ -775,7 +775,7 @@
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
     </row>
-    <row r="6" spans="1:19" ht="63.95">
+    <row r="6" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>25</v>
       </c>
@@ -795,7 +795,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:19">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="F7" s="3"/>
     </row>
   </sheetData>

</xml_diff>